<commit_message>
Fixes from agentic code review.
</commit_message>
<xml_diff>
--- a/sample-data/sample-run/Analysis.xlsx
+++ b/sample-data/sample-run/Analysis.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="262">
   <si>
     <t>Accident Period</t>
   </si>
@@ -405,7 +405,76 @@
     <t>Averages</t>
   </si>
   <si>
-    <t>Tail</t>
+    <t>11</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>83</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>107</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>131</t>
+  </si>
+  <si>
+    <t>143</t>
+  </si>
+  <si>
+    <t>155</t>
+  </si>
+  <si>
+    <t>167</t>
+  </si>
+  <si>
+    <t>179</t>
+  </si>
+  <si>
+    <t>191</t>
+  </si>
+  <si>
+    <t>203</t>
+  </si>
+  <si>
+    <t>215</t>
+  </si>
+  <si>
+    <t>227</t>
+  </si>
+  <si>
+    <t>239</t>
+  </si>
+  <si>
+    <t>251</t>
+  </si>
+  <si>
+    <t>263</t>
+  </si>
+  <si>
+    <t>275</t>
+  </si>
+  <si>
+    <t>287</t>
   </si>
   <si>
     <t>Average - All Years</t>
@@ -673,78 +742,6 @@
   </si>
   <si>
     <t>INCURRED SEVERITY</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>59</t>
-  </si>
-  <si>
-    <t>71</t>
-  </si>
-  <si>
-    <t>83</t>
-  </si>
-  <si>
-    <t>95</t>
-  </si>
-  <si>
-    <t>107</t>
-  </si>
-  <si>
-    <t>119</t>
-  </si>
-  <si>
-    <t>131</t>
-  </si>
-  <si>
-    <t>143</t>
-  </si>
-  <si>
-    <t>155</t>
-  </si>
-  <si>
-    <t>167</t>
-  </si>
-  <si>
-    <t>179</t>
-  </si>
-  <si>
-    <t>191</t>
-  </si>
-  <si>
-    <t>203</t>
-  </si>
-  <si>
-    <t>215</t>
-  </si>
-  <si>
-    <t>227</t>
-  </si>
-  <si>
-    <t>239</t>
-  </si>
-  <si>
-    <t>251</t>
-  </si>
-  <si>
-    <t>263</t>
-  </si>
-  <si>
-    <t>275</t>
-  </si>
-  <si>
-    <t>287</t>
   </si>
   <si>
     <t>PAID TO INCURRED</t>
@@ -1221,18 +1218,18 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1240,7 +1237,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1248,7 +1245,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1256,7 +1253,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1264,15 +1261,15 @@
         <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1280,7 +1277,7 @@
         <v>45</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1288,7 +1285,7 @@
         <v>46</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1296,7 +1293,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1304,7 +1301,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -1312,31 +1309,31 @@
         <v>44</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>213</v>
+        <v>236</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -1357,76 +1354,76 @@
       <c r="A1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="3">
+      <c r="B1" s="6">
         <v>11</v>
       </c>
-      <c r="C1" s="3">
+      <c r="C1" s="6">
         <v>23</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D1" s="6">
         <v>35</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="6">
         <v>47</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="6">
         <v>59</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="6">
         <v>71</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H1" s="6">
         <v>83</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I1" s="6">
         <v>95</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J1" s="6">
         <v>107</v>
       </c>
-      <c r="K1" s="3">
+      <c r="K1" s="6">
         <v>119</v>
       </c>
-      <c r="L1" s="3">
+      <c r="L1" s="6">
         <v>131</v>
       </c>
-      <c r="M1" s="3">
+      <c r="M1" s="6">
         <v>143</v>
       </c>
-      <c r="N1" s="3">
+      <c r="N1" s="6">
         <v>155</v>
       </c>
-      <c r="O1" s="3">
+      <c r="O1" s="6">
         <v>167</v>
       </c>
-      <c r="P1" s="3">
+      <c r="P1" s="6">
         <v>179</v>
       </c>
-      <c r="Q1" s="3">
+      <c r="Q1" s="6">
         <v>191</v>
       </c>
-      <c r="R1" s="3">
+      <c r="R1" s="6">
         <v>203</v>
       </c>
-      <c r="S1" s="3">
+      <c r="S1" s="6">
         <v>215</v>
       </c>
-      <c r="T1" s="3">
+      <c r="T1" s="6">
         <v>227</v>
       </c>
-      <c r="U1" s="3">
+      <c r="U1" s="6">
         <v>239</v>
       </c>
-      <c r="V1" s="3">
+      <c r="V1" s="6">
         <v>251</v>
       </c>
-      <c r="W1" s="3">
+      <c r="W1" s="6">
         <v>263</v>
       </c>
-      <c r="X1" s="3">
+      <c r="X1" s="6">
         <v>275</v>
       </c>
-      <c r="Y1" s="3">
+      <c r="Y1" s="6">
         <v>287</v>
       </c>
     </row>
@@ -4054,81 +4051,81 @@
         <v>124</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>77</v>
+        <v>125</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>79</v>
+        <v>127</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>81</v>
+        <v>129</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>83</v>
+        <v>131</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>84</v>
+        <v>132</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>85</v>
+        <v>133</v>
       </c>
       <c r="K52" s="3" t="s">
-        <v>86</v>
+        <v>134</v>
       </c>
       <c r="L52" s="3" t="s">
-        <v>87</v>
+        <v>135</v>
       </c>
       <c r="M52" s="3" t="s">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="N52" s="3" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="O52" s="3" t="s">
-        <v>90</v>
+        <v>138</v>
       </c>
       <c r="P52" s="3" t="s">
-        <v>91</v>
+        <v>139</v>
       </c>
       <c r="Q52" s="3" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="R52" s="3" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
       <c r="S52" s="3" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="T52" s="3" t="s">
-        <v>95</v>
+        <v>143</v>
       </c>
       <c r="U52" s="3" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="W52" s="3" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="X52" s="3" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="Y52" s="3" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
     </row>
     <row r="53" spans="1:25">
       <c r="A53" s="2" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="B53" s="6">
         <v>1.7435</v>
@@ -4203,7 +4200,7 @@
     </row>
     <row r="54" spans="1:25">
       <c r="A54" s="2" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B54" s="6">
         <v>1.6135</v>
@@ -4278,7 +4275,7 @@
     </row>
     <row r="55" spans="1:25">
       <c r="A55" s="2" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B55" s="6">
         <v>1.7265</v>
@@ -4353,7 +4350,7 @@
     </row>
     <row r="56" spans="1:25">
       <c r="A56" s="2" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="B56" s="6">
         <v>1.4593</v>
@@ -4428,7 +4425,7 @@
     </row>
     <row r="57" spans="1:25">
       <c r="A57" s="2" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="B57" s="6">
         <v>1.4891</v>
@@ -4503,7 +4500,7 @@
     </row>
     <row r="58" spans="1:25">
       <c r="A58" s="2" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="B58" s="6">
         <v>1.784</v>
@@ -4578,7 +4575,7 @@
     </row>
     <row r="59" spans="1:25">
       <c r="A59" s="2" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B59" s="6">
         <v>1.7024</v>
@@ -4653,7 +4650,7 @@
     </row>
     <row r="60" spans="1:25">
       <c r="A60" s="2" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="B60" s="6">
         <v>1.6456</v>
@@ -4728,7 +4725,7 @@
     </row>
     <row r="61" spans="1:25">
       <c r="A61" s="2" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="B61" s="6">
         <v>1.7774</v>
@@ -4803,7 +4800,7 @@
     </row>
     <row r="62" spans="1:25">
       <c r="A62" s="2" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="B62" s="6">
         <v>1.7371</v>
@@ -4878,7 +4875,7 @@
     </row>
     <row r="63" spans="1:25">
       <c r="A63" s="2" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="B63" s="6">
         <v>1.7238</v>
@@ -4953,7 +4950,7 @@
     </row>
     <row r="64" spans="1:25">
       <c r="A64" s="2" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="B64" s="6">
         <v>1.0888</v>
@@ -5028,7 +5025,7 @@
     </row>
     <row r="65" spans="1:25">
       <c r="A65" s="2" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="B65" s="6">
         <v>2.757</v>
@@ -5103,81 +5100,84 @@
     </row>
     <row r="67" spans="1:25">
       <c r="A67" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="L67" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="M67" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="N67" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="O67" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="P67" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B67" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K67" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="L67" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="M67" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="N67" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="O67" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="P67" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="Q67" s="3" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="R67" s="3" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
       <c r="S67" s="3" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="T67" s="3" t="s">
-        <v>95</v>
+        <v>143</v>
       </c>
       <c r="U67" s="3" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="W67" s="3" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="X67" s="3" t="s">
-        <v>99</v>
+        <v>147</v>
+      </c>
+      <c r="Y67" s="3" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="68" spans="1:25">
       <c r="A68" s="2" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="B68" s="6">
         <v>1.6456</v>
@@ -5251,77 +5251,77 @@
         <v>12</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>148</v>
+        <v>171</v>
       </c>
       <c r="J69" s="2" t="s">
-        <v>149</v>
+        <v>172</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
       <c r="M69" s="2" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="N69" s="2" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="O69" s="2" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="P69" s="2" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="Q69" s="2" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="R69" s="2" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="S69" s="2" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="T69" s="2" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="U69" s="2" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="V69" s="2" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="W69" s="2" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="X69" s="2"/>
       <c r="Y69" s="2"/>
     </row>
     <row r="71" spans="1:25">
       <c r="A71" s="2" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="B71" s="6">
         <v>1.6456</v>
@@ -5473,18 +5473,18 @@
     </row>
     <row r="74" spans="1:25">
       <c r="A74" s="2" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
     </row>
     <row r="75" spans="1:25" ht="240" customHeight="1">
       <c r="A75" s="2" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="9"/>
@@ -5512,76 +5512,76 @@
       <c r="A1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="3">
+      <c r="B1" s="6">
         <v>11</v>
       </c>
-      <c r="C1" s="3">
+      <c r="C1" s="6">
         <v>23</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D1" s="6">
         <v>35</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="6">
         <v>47</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="6">
         <v>59</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="6">
         <v>71</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H1" s="6">
         <v>83</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I1" s="6">
         <v>95</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J1" s="6">
         <v>107</v>
       </c>
-      <c r="K1" s="3">
+      <c r="K1" s="6">
         <v>119</v>
       </c>
-      <c r="L1" s="3">
+      <c r="L1" s="6">
         <v>131</v>
       </c>
-      <c r="M1" s="3">
+      <c r="M1" s="6">
         <v>143</v>
       </c>
-      <c r="N1" s="3">
+      <c r="N1" s="6">
         <v>155</v>
       </c>
-      <c r="O1" s="3">
+      <c r="O1" s="6">
         <v>167</v>
       </c>
-      <c r="P1" s="3">
+      <c r="P1" s="6">
         <v>179</v>
       </c>
-      <c r="Q1" s="3">
+      <c r="Q1" s="6">
         <v>191</v>
       </c>
-      <c r="R1" s="3">
+      <c r="R1" s="6">
         <v>203</v>
       </c>
-      <c r="S1" s="3">
+      <c r="S1" s="6">
         <v>215</v>
       </c>
-      <c r="T1" s="3">
+      <c r="T1" s="6">
         <v>227</v>
       </c>
-      <c r="U1" s="3">
+      <c r="U1" s="6">
         <v>239</v>
       </c>
-      <c r="V1" s="3">
+      <c r="V1" s="6">
         <v>251</v>
       </c>
-      <c r="W1" s="3">
+      <c r="W1" s="6">
         <v>263</v>
       </c>
-      <c r="X1" s="3">
+      <c r="X1" s="6">
         <v>275</v>
       </c>
-      <c r="Y1" s="3">
+      <c r="Y1" s="6">
         <v>287</v>
       </c>
     </row>
@@ -8209,81 +8209,81 @@
         <v>124</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>77</v>
+        <v>125</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>79</v>
+        <v>127</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>81</v>
+        <v>129</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>83</v>
+        <v>131</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>84</v>
+        <v>132</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>85</v>
+        <v>133</v>
       </c>
       <c r="K52" s="3" t="s">
-        <v>86</v>
+        <v>134</v>
       </c>
       <c r="L52" s="3" t="s">
-        <v>87</v>
+        <v>135</v>
       </c>
       <c r="M52" s="3" t="s">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="N52" s="3" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="O52" s="3" t="s">
-        <v>90</v>
+        <v>138</v>
       </c>
       <c r="P52" s="3" t="s">
-        <v>91</v>
+        <v>139</v>
       </c>
       <c r="Q52" s="3" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="R52" s="3" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
       <c r="S52" s="3" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="T52" s="3" t="s">
-        <v>95</v>
+        <v>143</v>
       </c>
       <c r="U52" s="3" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="W52" s="3" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="X52" s="3" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="Y52" s="3" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
     </row>
     <row r="53" spans="1:25">
       <c r="A53" s="2" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="B53" s="6">
         <v>2.4979</v>
@@ -8358,7 +8358,7 @@
     </row>
     <row r="54" spans="1:25">
       <c r="A54" s="2" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B54" s="6">
         <v>2.4566</v>
@@ -8433,7 +8433,7 @@
     </row>
     <row r="55" spans="1:25">
       <c r="A55" s="2" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B55" s="6">
         <v>2.4952</v>
@@ -8508,7 +8508,7 @@
     </row>
     <row r="56" spans="1:25">
       <c r="A56" s="2" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="B56" s="6">
         <v>2.5643</v>
@@ -8583,7 +8583,7 @@
     </row>
     <row r="57" spans="1:25">
       <c r="A57" s="2" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="B57" s="6">
         <v>2.6286</v>
@@ -8658,7 +8658,7 @@
     </row>
     <row r="58" spans="1:25">
       <c r="A58" s="2" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="B58" s="6">
         <v>2.5842</v>
@@ -8733,7 +8733,7 @@
     </row>
     <row r="59" spans="1:25">
       <c r="A59" s="2" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B59" s="6">
         <v>2.6232</v>
@@ -8808,7 +8808,7 @@
     </row>
     <row r="60" spans="1:25">
       <c r="A60" s="2" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="B60" s="6">
         <v>2.5525</v>
@@ -8883,7 +8883,7 @@
     </row>
     <row r="61" spans="1:25">
       <c r="A61" s="2" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="B61" s="6">
         <v>2.4862</v>
@@ -8958,7 +8958,7 @@
     </row>
     <row r="62" spans="1:25">
       <c r="A62" s="2" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="B62" s="6">
         <v>2.482</v>
@@ -9033,7 +9033,7 @@
     </row>
     <row r="63" spans="1:25">
       <c r="A63" s="2" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="B63" s="6">
         <v>2.4762</v>
@@ -9108,7 +9108,7 @@
     </row>
     <row r="64" spans="1:25">
       <c r="A64" s="2" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="B64" s="6">
         <v>1.7371</v>
@@ -9183,7 +9183,7 @@
     </row>
     <row r="65" spans="1:25">
       <c r="A65" s="2" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="B65" s="6">
         <v>3.3152</v>
@@ -9258,81 +9258,84 @@
     </row>
     <row r="67" spans="1:25">
       <c r="A67" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="L67" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="M67" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="N67" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="O67" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="P67" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B67" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K67" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="L67" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="M67" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="N67" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="O67" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="P67" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="Q67" s="3" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="R67" s="3" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
       <c r="S67" s="3" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="T67" s="3" t="s">
-        <v>95</v>
+        <v>143</v>
       </c>
       <c r="U67" s="3" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="W67" s="3" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="X67" s="3" t="s">
-        <v>99</v>
+        <v>147</v>
+      </c>
+      <c r="Y67" s="3" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="68" spans="1:25">
       <c r="A68" s="2" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="B68" s="6">
         <v>2.5525</v>
@@ -9406,77 +9409,77 @@
         <v>12</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="J69" s="2" t="s">
-        <v>176</v>
+        <v>199</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="M69" s="2" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
       <c r="N69" s="2" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="O69" s="2" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
       <c r="P69" s="2" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="Q69" s="2" t="s">
-        <v>183</v>
+        <v>206</v>
       </c>
       <c r="R69" s="2" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
       <c r="S69" s="2" t="s">
-        <v>185</v>
+        <v>208</v>
       </c>
       <c r="T69" s="2" t="s">
-        <v>186</v>
+        <v>209</v>
       </c>
       <c r="U69" s="2" t="s">
-        <v>187</v>
+        <v>210</v>
       </c>
       <c r="V69" s="2" t="s">
-        <v>188</v>
+        <v>211</v>
       </c>
       <c r="W69" s="2" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="X69" s="2"/>
       <c r="Y69" s="2"/>
     </row>
     <row r="71" spans="1:25">
       <c r="A71" s="2" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="B71" s="6">
         <v>2.5525</v>
@@ -9628,18 +9631,18 @@
     </row>
     <row r="74" spans="1:25">
       <c r="A74" s="2" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
     </row>
     <row r="75" spans="1:25" ht="270" customHeight="1">
       <c r="A75" s="2" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="9"/>
@@ -9667,76 +9670,76 @@
       <c r="A1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="3">
+      <c r="B1" s="6">
         <v>11</v>
       </c>
-      <c r="C1" s="3">
+      <c r="C1" s="6">
         <v>23</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D1" s="6">
         <v>35</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="6">
         <v>47</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="6">
         <v>59</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="6">
         <v>71</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H1" s="6">
         <v>83</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I1" s="6">
         <v>95</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J1" s="6">
         <v>107</v>
       </c>
-      <c r="K1" s="3">
+      <c r="K1" s="6">
         <v>119</v>
       </c>
-      <c r="L1" s="3">
+      <c r="L1" s="6">
         <v>131</v>
       </c>
-      <c r="M1" s="3">
+      <c r="M1" s="6">
         <v>143</v>
       </c>
-      <c r="N1" s="3">
+      <c r="N1" s="6">
         <v>155</v>
       </c>
-      <c r="O1" s="3">
+      <c r="O1" s="6">
         <v>167</v>
       </c>
-      <c r="P1" s="3">
+      <c r="P1" s="6">
         <v>179</v>
       </c>
-      <c r="Q1" s="3">
+      <c r="Q1" s="6">
         <v>191</v>
       </c>
-      <c r="R1" s="3">
+      <c r="R1" s="6">
         <v>203</v>
       </c>
-      <c r="S1" s="3">
+      <c r="S1" s="6">
         <v>215</v>
       </c>
-      <c r="T1" s="3">
+      <c r="T1" s="6">
         <v>227</v>
       </c>
-      <c r="U1" s="3">
+      <c r="U1" s="6">
         <v>239</v>
       </c>
-      <c r="V1" s="3">
+      <c r="V1" s="6">
         <v>251</v>
       </c>
-      <c r="W1" s="3">
+      <c r="W1" s="6">
         <v>263</v>
       </c>
-      <c r="X1" s="3">
+      <c r="X1" s="6">
         <v>275</v>
       </c>
-      <c r="Y1" s="3">
+      <c r="Y1" s="6">
         <v>287</v>
       </c>
     </row>
@@ -12364,81 +12367,81 @@
         <v>124</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>77</v>
+        <v>125</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>79</v>
+        <v>127</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>81</v>
+        <v>129</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>83</v>
+        <v>131</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>84</v>
+        <v>132</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>85</v>
+        <v>133</v>
       </c>
       <c r="K52" s="3" t="s">
-        <v>86</v>
+        <v>134</v>
       </c>
       <c r="L52" s="3" t="s">
-        <v>87</v>
+        <v>135</v>
       </c>
       <c r="M52" s="3" t="s">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="N52" s="3" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="O52" s="3" t="s">
-        <v>90</v>
+        <v>138</v>
       </c>
       <c r="P52" s="3" t="s">
-        <v>91</v>
+        <v>139</v>
       </c>
       <c r="Q52" s="3" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="R52" s="3" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
       <c r="S52" s="3" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="T52" s="3" t="s">
-        <v>95</v>
+        <v>143</v>
       </c>
       <c r="U52" s="3" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="V52" s="3" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="W52" s="3" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="X52" s="3" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="Y52" s="3" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
     </row>
     <row r="53" spans="1:25">
       <c r="A53" s="2" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="B53" s="6">
         <v>1.0679</v>
@@ -12513,7 +12516,7 @@
     </row>
     <row r="54" spans="1:25">
       <c r="A54" s="2" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B54" s="6">
         <v>1.0617</v>
@@ -12588,7 +12591,7 @@
     </row>
     <row r="55" spans="1:25">
       <c r="A55" s="2" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B55" s="6">
         <v>1.0676</v>
@@ -12663,7 +12666,7 @@
     </row>
     <row r="56" spans="1:25">
       <c r="A56" s="2" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="B56" s="6">
         <v>1.133</v>
@@ -12738,7 +12741,7 @@
     </row>
     <row r="57" spans="1:25">
       <c r="A57" s="2" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="B57" s="6">
         <v>1.133</v>
@@ -12813,7 +12816,7 @@
     </row>
     <row r="58" spans="1:25">
       <c r="A58" s="2" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="B58" s="6">
         <v>1.1204</v>
@@ -12888,7 +12891,7 @@
     </row>
     <row r="59" spans="1:25">
       <c r="A59" s="2" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B59" s="6">
         <v>1.118</v>
@@ -12963,7 +12966,7 @@
     </row>
     <row r="60" spans="1:25">
       <c r="A60" s="2" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="B60" s="6">
         <v>1.133</v>
@@ -13038,7 +13041,7 @@
     </row>
     <row r="61" spans="1:25">
       <c r="A61" s="2" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="B61" s="6">
         <v>1.1009</v>
@@ -13113,7 +13116,7 @@
     </row>
     <row r="62" spans="1:25">
       <c r="A62" s="2" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="B62" s="6">
         <v>1.0962</v>
@@ -13188,7 +13191,7 @@
     </row>
     <row r="63" spans="1:25">
       <c r="A63" s="2" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="B63" s="6">
         <v>1.1041</v>
@@ -13263,7 +13266,7 @@
     </row>
     <row r="64" spans="1:25">
       <c r="A64" s="2" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="B64" s="6">
         <v>1</v>
@@ -13338,7 +13341,7 @@
     </row>
     <row r="65" spans="1:25">
       <c r="A65" s="2" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="B65" s="6">
         <v>1.1429</v>
@@ -13413,81 +13416,84 @@
     </row>
     <row r="67" spans="1:25">
       <c r="A67" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="L67" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="M67" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="N67" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="O67" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="P67" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B67" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K67" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="L67" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="M67" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="N67" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="O67" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="P67" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="Q67" s="3" t="s">
-        <v>92</v>
+        <v>140</v>
       </c>
       <c r="R67" s="3" t="s">
-        <v>93</v>
+        <v>141</v>
       </c>
       <c r="S67" s="3" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="T67" s="3" t="s">
-        <v>95</v>
+        <v>143</v>
       </c>
       <c r="U67" s="3" t="s">
-        <v>96</v>
+        <v>144</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>97</v>
+        <v>145</v>
       </c>
       <c r="W67" s="3" t="s">
-        <v>98</v>
+        <v>146</v>
       </c>
       <c r="X67" s="3" t="s">
-        <v>99</v>
+        <v>147</v>
+      </c>
+      <c r="Y67" s="3" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="68" spans="1:25">
       <c r="A68" s="2" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="B68" s="6">
         <v>1.133</v>
@@ -13563,79 +13569,79 @@
         <v>12</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>192</v>
+        <v>215</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>194</v>
+        <v>217</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
       <c r="J69" s="2" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>200</v>
+        <v>223</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>201</v>
+        <v>224</v>
       </c>
       <c r="M69" s="2" t="s">
-        <v>202</v>
+        <v>225</v>
       </c>
       <c r="N69" s="2" t="s">
-        <v>203</v>
+        <v>226</v>
       </c>
       <c r="O69" s="2" t="s">
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="P69" s="2" t="s">
-        <v>205</v>
+        <v>228</v>
       </c>
       <c r="Q69" s="2" t="s">
-        <v>206</v>
+        <v>229</v>
       </c>
       <c r="R69" s="2" t="s">
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="S69" s="2" t="s">
-        <v>207</v>
+        <v>230</v>
       </c>
       <c r="T69" s="2" t="s">
-        <v>208</v>
+        <v>231</v>
       </c>
       <c r="U69" s="2" t="s">
-        <v>209</v>
+        <v>232</v>
       </c>
       <c r="V69" s="2" t="s">
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="W69" s="2" t="s">
-        <v>210</v>
+        <v>233</v>
       </c>
       <c r="X69" s="2" t="s">
-        <v>211</v>
+        <v>234</v>
       </c>
       <c r="Y69" s="2"/>
     </row>
     <row r="71" spans="1:25">
       <c r="A71" s="2" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="B71" s="6">
         <v>1.133</v>
@@ -13787,18 +13793,18 @@
     </row>
     <row r="74" spans="1:25">
       <c r="A74" s="2" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
     </row>
     <row r="75" spans="1:25" ht="285" customHeight="1">
       <c r="A75" s="2" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="9"/>
@@ -13826,7 +13832,7 @@
         <v>75</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>213</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -14037,7 +14043,7 @@
   <sheetData>
     <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>237</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -14069,76 +14075,76 @@
         <v>75</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>216</v>
+        <v>126</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>217</v>
+        <v>127</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>219</v>
+        <v>129</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>223</v>
+        <v>133</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>224</v>
+        <v>134</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>225</v>
+        <v>135</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>226</v>
+        <v>136</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>227</v>
+        <v>137</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>228</v>
+        <v>138</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>229</v>
+        <v>139</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="R2" s="10" t="s">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>232</v>
+        <v>142</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>233</v>
+        <v>143</v>
       </c>
       <c r="U2" s="10" t="s">
-        <v>234</v>
+        <v>144</v>
       </c>
       <c r="V2" s="10" t="s">
-        <v>235</v>
+        <v>145</v>
       </c>
       <c r="W2" s="10" t="s">
-        <v>236</v>
+        <v>146</v>
       </c>
       <c r="X2" s="10" t="s">
-        <v>237</v>
+        <v>147</v>
       </c>
       <c r="Y2" s="10" t="s">
-        <v>238</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -15163,7 +15169,7 @@
     </row>
     <row r="28" spans="1:25">
       <c r="A28" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -15195,76 +15201,76 @@
         <v>75</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>216</v>
+        <v>126</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>217</v>
+        <v>127</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>219</v>
+        <v>129</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
       <c r="J29" s="10" t="s">
-        <v>223</v>
+        <v>133</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>224</v>
+        <v>134</v>
       </c>
       <c r="L29" s="10" t="s">
-        <v>225</v>
+        <v>135</v>
       </c>
       <c r="M29" s="10" t="s">
-        <v>226</v>
+        <v>136</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>227</v>
+        <v>137</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>228</v>
+        <v>138</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>229</v>
+        <v>139</v>
       </c>
       <c r="Q29" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="R29" s="10" t="s">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="S29" s="10" t="s">
-        <v>232</v>
+        <v>142</v>
       </c>
       <c r="T29" s="10" t="s">
-        <v>233</v>
+        <v>143</v>
       </c>
       <c r="U29" s="10" t="s">
-        <v>234</v>
+        <v>144</v>
       </c>
       <c r="V29" s="10" t="s">
-        <v>235</v>
+        <v>145</v>
       </c>
       <c r="W29" s="10" t="s">
-        <v>236</v>
+        <v>146</v>
       </c>
       <c r="X29" s="10" t="s">
-        <v>237</v>
+        <v>147</v>
       </c>
       <c r="Y29" s="10" t="s">
-        <v>238</v>
+        <v>148</v>
       </c>
     </row>
     <row r="30" spans="1:25">
@@ -16289,7 +16295,7 @@
     </row>
     <row r="55" spans="1:25">
       <c r="A55" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -16321,76 +16327,76 @@
         <v>75</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>216</v>
+        <v>126</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>217</v>
+        <v>127</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="F56" s="10" t="s">
-        <v>219</v>
+        <v>129</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="H56" s="10" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
       <c r="J56" s="10" t="s">
-        <v>223</v>
+        <v>133</v>
       </c>
       <c r="K56" s="10" t="s">
-        <v>224</v>
+        <v>134</v>
       </c>
       <c r="L56" s="10" t="s">
-        <v>225</v>
+        <v>135</v>
       </c>
       <c r="M56" s="10" t="s">
-        <v>226</v>
+        <v>136</v>
       </c>
       <c r="N56" s="10" t="s">
-        <v>227</v>
+        <v>137</v>
       </c>
       <c r="O56" s="10" t="s">
-        <v>228</v>
+        <v>138</v>
       </c>
       <c r="P56" s="10" t="s">
-        <v>229</v>
+        <v>139</v>
       </c>
       <c r="Q56" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="R56" s="10" t="s">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="S56" s="10" t="s">
-        <v>232</v>
+        <v>142</v>
       </c>
       <c r="T56" s="10" t="s">
-        <v>233</v>
+        <v>143</v>
       </c>
       <c r="U56" s="10" t="s">
-        <v>234</v>
+        <v>144</v>
       </c>
       <c r="V56" s="10" t="s">
-        <v>235</v>
+        <v>145</v>
       </c>
       <c r="W56" s="10" t="s">
-        <v>236</v>
+        <v>146</v>
       </c>
       <c r="X56" s="10" t="s">
-        <v>237</v>
+        <v>147</v>
       </c>
       <c r="Y56" s="10" t="s">
-        <v>238</v>
+        <v>148</v>
       </c>
     </row>
     <row r="57" spans="1:25">
@@ -17415,7 +17421,7 @@
     </row>
     <row r="82" spans="1:25">
       <c r="A82" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -17447,76 +17453,76 @@
         <v>75</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>216</v>
+        <v>126</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>217</v>
+        <v>127</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="F83" s="10" t="s">
-        <v>219</v>
+        <v>129</v>
       </c>
       <c r="G83" s="10" t="s">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="I83" s="10" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
       <c r="J83" s="10" t="s">
-        <v>223</v>
+        <v>133</v>
       </c>
       <c r="K83" s="10" t="s">
-        <v>224</v>
+        <v>134</v>
       </c>
       <c r="L83" s="10" t="s">
-        <v>225</v>
+        <v>135</v>
       </c>
       <c r="M83" s="10" t="s">
-        <v>226</v>
+        <v>136</v>
       </c>
       <c r="N83" s="10" t="s">
-        <v>227</v>
+        <v>137</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>228</v>
+        <v>138</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>229</v>
+        <v>139</v>
       </c>
       <c r="Q83" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="R83" s="10" t="s">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="S83" s="10" t="s">
-        <v>232</v>
+        <v>142</v>
       </c>
       <c r="T83" s="10" t="s">
-        <v>233</v>
+        <v>143</v>
       </c>
       <c r="U83" s="10" t="s">
-        <v>234</v>
+        <v>144</v>
       </c>
       <c r="V83" s="10" t="s">
-        <v>235</v>
+        <v>145</v>
       </c>
       <c r="W83" s="10" t="s">
-        <v>236</v>
+        <v>146</v>
       </c>
       <c r="X83" s="10" t="s">
-        <v>237</v>
+        <v>147</v>
       </c>
       <c r="Y83" s="10" t="s">
-        <v>238</v>
+        <v>148</v>
       </c>
     </row>
     <row r="84" spans="1:25">
@@ -18541,7 +18547,7 @@
     </row>
     <row r="109" spans="1:25">
       <c r="A109" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -18573,76 +18579,76 @@
         <v>75</v>
       </c>
       <c r="B110" s="10" t="s">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C110" s="10" t="s">
-        <v>216</v>
+        <v>126</v>
       </c>
       <c r="D110" s="10" t="s">
-        <v>217</v>
+        <v>127</v>
       </c>
       <c r="E110" s="10" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="F110" s="10" t="s">
-        <v>219</v>
+        <v>129</v>
       </c>
       <c r="G110" s="10" t="s">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="H110" s="10" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="I110" s="10" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
       <c r="J110" s="10" t="s">
-        <v>223</v>
+        <v>133</v>
       </c>
       <c r="K110" s="10" t="s">
-        <v>224</v>
+        <v>134</v>
       </c>
       <c r="L110" s="10" t="s">
-        <v>225</v>
+        <v>135</v>
       </c>
       <c r="M110" s="10" t="s">
-        <v>226</v>
+        <v>136</v>
       </c>
       <c r="N110" s="10" t="s">
-        <v>227</v>
+        <v>137</v>
       </c>
       <c r="O110" s="10" t="s">
-        <v>228</v>
+        <v>138</v>
       </c>
       <c r="P110" s="10" t="s">
-        <v>229</v>
+        <v>139</v>
       </c>
       <c r="Q110" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="R110" s="10" t="s">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="S110" s="10" t="s">
-        <v>232</v>
+        <v>142</v>
       </c>
       <c r="T110" s="10" t="s">
-        <v>233</v>
+        <v>143</v>
       </c>
       <c r="U110" s="10" t="s">
-        <v>234</v>
+        <v>144</v>
       </c>
       <c r="V110" s="10" t="s">
-        <v>235</v>
+        <v>145</v>
       </c>
       <c r="W110" s="10" t="s">
-        <v>236</v>
+        <v>146</v>
       </c>
       <c r="X110" s="10" t="s">
-        <v>237</v>
+        <v>147</v>
       </c>
       <c r="Y110" s="10" t="s">
-        <v>238</v>
+        <v>148</v>
       </c>
     </row>
     <row r="111" spans="1:25">
@@ -19667,7 +19673,7 @@
     </row>
     <row r="136" spans="1:25">
       <c r="A136" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -19699,76 +19705,76 @@
         <v>75</v>
       </c>
       <c r="B137" s="10" t="s">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C137" s="10" t="s">
-        <v>216</v>
+        <v>126</v>
       </c>
       <c r="D137" s="10" t="s">
-        <v>217</v>
+        <v>127</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="F137" s="10" t="s">
-        <v>219</v>
+        <v>129</v>
       </c>
       <c r="G137" s="10" t="s">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="H137" s="10" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="I137" s="10" t="s">
-        <v>222</v>
+        <v>132</v>
       </c>
       <c r="J137" s="10" t="s">
-        <v>223</v>
+        <v>133</v>
       </c>
       <c r="K137" s="10" t="s">
-        <v>224</v>
+        <v>134</v>
       </c>
       <c r="L137" s="10" t="s">
-        <v>225</v>
+        <v>135</v>
       </c>
       <c r="M137" s="10" t="s">
-        <v>226</v>
+        <v>136</v>
       </c>
       <c r="N137" s="10" t="s">
-        <v>227</v>
+        <v>137</v>
       </c>
       <c r="O137" s="10" t="s">
-        <v>228</v>
+        <v>138</v>
       </c>
       <c r="P137" s="10" t="s">
-        <v>229</v>
+        <v>139</v>
       </c>
       <c r="Q137" s="10" t="s">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="R137" s="10" t="s">
-        <v>231</v>
+        <v>141</v>
       </c>
       <c r="S137" s="10" t="s">
-        <v>232</v>
+        <v>142</v>
       </c>
       <c r="T137" s="10" t="s">
-        <v>233</v>
+        <v>143</v>
       </c>
       <c r="U137" s="10" t="s">
-        <v>234</v>
+        <v>144</v>
       </c>
       <c r="V137" s="10" t="s">
-        <v>235</v>
+        <v>145</v>
       </c>
       <c r="W137" s="10" t="s">
-        <v>236</v>
+        <v>146</v>
       </c>
       <c r="X137" s="10" t="s">
-        <v>237</v>
+        <v>147</v>
       </c>
       <c r="Y137" s="10" t="s">
-        <v>238</v>
+        <v>148</v>
       </c>
     </row>
     <row r="138" spans="1:25">
@@ -21165,7 +21171,7 @@
     </row>
     <row r="28" spans="1:25">
       <c r="A28" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -22291,7 +22297,7 @@
     </row>
     <row r="55" spans="1:25">
       <c r="A55" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -23417,7 +23423,7 @@
     </row>
     <row r="82" spans="1:25">
       <c r="A82" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -24543,7 +24549,7 @@
     </row>
     <row r="109" spans="1:25">
       <c r="A109" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -25669,7 +25675,7 @@
     </row>
     <row r="136" spans="1:25">
       <c r="A136" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>

</xml_diff>